<commit_message>
chore: refactor import student
</commit_message>
<xml_diff>
--- a/src/test/resources/mock/test-grade-import.xlsx
+++ b/src/test/resources/mock/test-grade-import.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>ref</t>
   </si>
@@ -27,7 +27,13 @@
     <t>STD21002</t>
   </si>
   <si>
-    <t>STD21003</t>
+    <t>STD21009</t>
+  </si>
+  <si>
+    <t>STD21010</t>
+  </si>
+  <si>
+    <t>STD23009</t>
   </si>
 </sst>
 </file>
@@ -62,10 +68,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -589,8 +598,34 @@
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>9.5</v>
+    </row>
+    <row r="4" ht="14.25">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="B5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: switch grade import to front-all (remove event worker)
</commit_message>
<xml_diff>
--- a/src/test/resources/mock/test-grade-import.xlsx
+++ b/src/test/resources/mock/test-grade-import.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>ref</t>
   </si>
@@ -28,6 +28,12 @@
   </si>
   <si>
     <t>STD21003</t>
+  </si>
+  <si>
+    <t>STD21009</t>
+  </si>
+  <si>
+    <t>STD21011</t>
   </si>
 </sst>
 </file>
@@ -62,10 +68,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -589,8 +598,42 @@
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>9.5</v>
+    </row>
+    <row r="4" ht="14.25">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="B5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: udpate grade via excel file
</commit_message>
<xml_diff>
--- a/src/test/resources/mock/test-grade-import.xlsx
+++ b/src/test/resources/mock/test-grade-import.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ref</t>
   </si>
@@ -24,7 +24,10 @@
     <t>score</t>
   </si>
   <si>
-    <t>STD21002</t>
+    <t>STD22031</t>
+  </si>
+  <si>
+    <t>STD22033</t>
   </si>
   <si>
     <t>STD21003</t>
@@ -68,7 +71,11 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -587,37 +594,37 @@
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>12</v>
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="B3" s="4">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
+      <c r="A4" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
         <v>13</v>
       </c>
     </row>
-    <row r="5" ht="14.25">
-      <c r="B5">
+    <row r="6" ht="14.25">
+      <c r="B6">
         <v>12</v>
-      </c>
-    </row>
-    <row r="6" ht="14.25">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6">
-        <v>23</v>
       </c>
     </row>
     <row r="7" ht="14.25">
@@ -625,14 +632,22 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>-1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B8">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
         <v>13</v>
       </c>
     </row>

</xml_diff>